<commit_message>
Actualizacion de notas y tablas de resultados separadas
</commit_message>
<xml_diff>
--- a/backend/database/Seguidores_Primer_Modulo.xlsx
+++ b/backend/database/Seguidores_Primer_Modulo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/24b0972e82577483/CLOUDGER/DOCKER/NOTAS_MOVI_APP/notasseguidores/app/backend/database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="47" documentId="8_{CB1EA7B0-2F00-435E-A2E5-997CDBADE84E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E6E607AA-ACC9-4177-B527-A4A69FD571D7}"/>
+  <xr:revisionPtr revIDLastSave="49" documentId="8_{CB1EA7B0-2F00-435E-A2E5-997CDBADE84E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B223C419-B485-4544-838F-12A10B0266E9}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5BEBD1D6-3E86-4F2C-B143-CBE730185EB4}"/>
   </bookViews>
@@ -1655,7 +1655,7 @@
         <v>10</v>
       </c>
       <c r="I2">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J2">
         <v>10</v>
@@ -1706,7 +1706,7 @@
         <v>10</v>
       </c>
       <c r="I3">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J3">
         <v>10</v>
@@ -1728,7 +1728,7 @@
       </c>
       <c r="P3">
         <f t="shared" ref="P3:P66" si="0">ROUNDUP(AVERAGE(D3:O3),0)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
@@ -1757,7 +1757,7 @@
         <v>10</v>
       </c>
       <c r="I4">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J4">
         <v>10</v>
@@ -1808,7 +1808,7 @@
         <v>10</v>
       </c>
       <c r="I5">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J5">
         <v>10</v>
@@ -1859,7 +1859,7 @@
         <v>10</v>
       </c>
       <c r="I6">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J6">
         <v>10</v>
@@ -1881,7 +1881,7 @@
       </c>
       <c r="P6">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
@@ -1910,7 +1910,7 @@
         <v>10</v>
       </c>
       <c r="I7">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J7">
         <v>10</v>
@@ -1932,7 +1932,7 @@
       </c>
       <c r="P7">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
@@ -1961,7 +1961,7 @@
         <v>10</v>
       </c>
       <c r="I8">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J8">
         <v>10</v>
@@ -2012,7 +2012,7 @@
         <v>10</v>
       </c>
       <c r="I9">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J9">
         <v>10</v>
@@ -2034,7 +2034,7 @@
       </c>
       <c r="P9">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
@@ -2063,7 +2063,7 @@
         <v>10</v>
       </c>
       <c r="I10">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J10">
         <v>10</v>
@@ -2085,7 +2085,7 @@
       </c>
       <c r="P10">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
@@ -2114,7 +2114,7 @@
         <v>10</v>
       </c>
       <c r="I11">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J11">
         <v>10</v>
@@ -2136,7 +2136,7 @@
       </c>
       <c r="P11">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
@@ -2165,7 +2165,7 @@
         <v>10</v>
       </c>
       <c r="I12">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J12">
         <v>10</v>
@@ -2216,7 +2216,7 @@
         <v>10</v>
       </c>
       <c r="I13">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J13">
         <v>10</v>
@@ -2238,7 +2238,7 @@
       </c>
       <c r="P13">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
@@ -2267,7 +2267,7 @@
         <v>10</v>
       </c>
       <c r="I14">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J14">
         <v>10</v>
@@ -2289,7 +2289,7 @@
       </c>
       <c r="P14">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
@@ -2318,7 +2318,7 @@
         <v>10</v>
       </c>
       <c r="I15">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J15">
         <v>10</v>
@@ -2369,7 +2369,7 @@
         <v>10</v>
       </c>
       <c r="I16">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J16">
         <v>0</v>
@@ -2391,7 +2391,7 @@
       </c>
       <c r="P16">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.25">
@@ -2420,7 +2420,7 @@
         <v>10</v>
       </c>
       <c r="I17">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J17">
         <v>10</v>
@@ -2442,7 +2442,7 @@
       </c>
       <c r="P17">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
@@ -2471,7 +2471,7 @@
         <v>10</v>
       </c>
       <c r="I18">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J18">
         <v>10</v>
@@ -2522,7 +2522,7 @@
         <v>10</v>
       </c>
       <c r="I19">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J19">
         <v>0</v>
@@ -2544,7 +2544,7 @@
       </c>
       <c r="P19">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
@@ -2573,7 +2573,7 @@
         <v>10</v>
       </c>
       <c r="I20">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J20">
         <v>10</v>
@@ -2595,7 +2595,7 @@
       </c>
       <c r="P20">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.25">
@@ -2624,7 +2624,7 @@
         <v>0</v>
       </c>
       <c r="I21">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J21">
         <v>0</v>
@@ -2646,7 +2646,7 @@
       </c>
       <c r="P21">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.25">
@@ -2675,7 +2675,7 @@
         <v>10</v>
       </c>
       <c r="I22">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J22">
         <v>0</v>
@@ -2697,7 +2697,7 @@
       </c>
       <c r="P22">
         <f t="shared" si="0"/>
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.25">
@@ -2726,7 +2726,7 @@
         <v>10</v>
       </c>
       <c r="I23">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J23">
         <v>10</v>
@@ -2777,7 +2777,7 @@
         <v>10</v>
       </c>
       <c r="I24">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J24">
         <v>10</v>
@@ -2828,7 +2828,7 @@
         <v>10</v>
       </c>
       <c r="I25">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J25">
         <v>10</v>
@@ -2879,7 +2879,7 @@
         <v>10</v>
       </c>
       <c r="I26">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J26">
         <v>10</v>
@@ -2901,7 +2901,7 @@
       </c>
       <c r="P26">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.25">
@@ -2930,7 +2930,7 @@
         <v>10</v>
       </c>
       <c r="I27">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J27">
         <v>10</v>
@@ -2952,7 +2952,7 @@
       </c>
       <c r="P27">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.25">
@@ -2981,7 +2981,7 @@
         <v>10</v>
       </c>
       <c r="I28">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J28">
         <v>10</v>
@@ -3003,7 +3003,7 @@
       </c>
       <c r="P28">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="29" spans="1:16" x14ac:dyDescent="0.25">
@@ -3032,7 +3032,7 @@
         <v>10</v>
       </c>
       <c r="I29">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J29">
         <v>10</v>
@@ -3054,7 +3054,7 @@
       </c>
       <c r="P29">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.25">
@@ -3083,7 +3083,7 @@
         <v>10</v>
       </c>
       <c r="I30">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J30">
         <v>0</v>
@@ -3105,7 +3105,7 @@
       </c>
       <c r="P30">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.25">
@@ -3134,7 +3134,7 @@
         <v>10</v>
       </c>
       <c r="I31">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J31">
         <v>10</v>
@@ -3236,7 +3236,7 @@
         <v>10</v>
       </c>
       <c r="I33">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J33">
         <v>10</v>
@@ -3258,7 +3258,7 @@
       </c>
       <c r="P33">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.25">
@@ -3287,7 +3287,7 @@
         <v>10</v>
       </c>
       <c r="I34">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J34">
         <v>10</v>
@@ -3338,7 +3338,7 @@
         <v>10</v>
       </c>
       <c r="I35">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J35">
         <v>10</v>
@@ -3389,7 +3389,7 @@
         <v>10</v>
       </c>
       <c r="I36">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J36">
         <v>10</v>
@@ -3440,7 +3440,7 @@
         <v>10</v>
       </c>
       <c r="I37">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J37">
         <v>10</v>
@@ -3491,7 +3491,7 @@
         <v>10</v>
       </c>
       <c r="I38">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J38">
         <v>10</v>
@@ -3513,7 +3513,7 @@
       </c>
       <c r="P38">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.25">
@@ -3542,7 +3542,7 @@
         <v>10</v>
       </c>
       <c r="I39">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J39">
         <v>10</v>
@@ -3564,7 +3564,7 @@
       </c>
       <c r="P39">
         <f t="shared" si="0"/>
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.25">
@@ -3593,7 +3593,7 @@
         <v>10</v>
       </c>
       <c r="I40">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J40">
         <v>10</v>
@@ -3644,7 +3644,7 @@
         <v>10</v>
       </c>
       <c r="I41">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J41">
         <v>10</v>
@@ -3666,7 +3666,7 @@
       </c>
       <c r="P41">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="42" spans="1:16" x14ac:dyDescent="0.25">
@@ -3695,7 +3695,7 @@
         <v>10</v>
       </c>
       <c r="I42">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J42">
         <v>10</v>
@@ -3717,7 +3717,7 @@
       </c>
       <c r="P42">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="43" spans="1:16" x14ac:dyDescent="0.25">
@@ -3746,7 +3746,7 @@
         <v>10</v>
       </c>
       <c r="I43">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J43">
         <v>10</v>
@@ -3768,7 +3768,7 @@
       </c>
       <c r="P43">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="44" spans="1:16" x14ac:dyDescent="0.25">
@@ -3797,7 +3797,7 @@
         <v>10</v>
       </c>
       <c r="I44">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J44">
         <v>10</v>
@@ -3819,7 +3819,7 @@
       </c>
       <c r="P44">
         <f t="shared" si="0"/>
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="45" spans="1:16" x14ac:dyDescent="0.25">
@@ -3848,7 +3848,7 @@
         <v>10</v>
       </c>
       <c r="I45">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J45">
         <v>10</v>
@@ -3870,7 +3870,7 @@
       </c>
       <c r="P45">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="46" spans="1:16" x14ac:dyDescent="0.25">
@@ -3899,7 +3899,7 @@
         <v>0</v>
       </c>
       <c r="I46">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J46">
         <v>0</v>
@@ -3921,7 +3921,7 @@
       </c>
       <c r="P46">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47" spans="1:16" x14ac:dyDescent="0.25">
@@ -3950,7 +3950,7 @@
         <v>10</v>
       </c>
       <c r="I47">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J47">
         <v>10</v>
@@ -4001,7 +4001,7 @@
         <v>10</v>
       </c>
       <c r="I48">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J48">
         <v>0</v>
@@ -4023,7 +4023,7 @@
       </c>
       <c r="P48">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="49" spans="1:16" x14ac:dyDescent="0.25">
@@ -4052,7 +4052,7 @@
         <v>10</v>
       </c>
       <c r="I49">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J49">
         <v>10</v>
@@ -4074,7 +4074,7 @@
       </c>
       <c r="P49">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="50" spans="1:16" x14ac:dyDescent="0.25">
@@ -4103,7 +4103,7 @@
         <v>10</v>
       </c>
       <c r="I50">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J50">
         <v>10</v>
@@ -4154,7 +4154,7 @@
         <v>10</v>
       </c>
       <c r="I51">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J51">
         <v>0</v>
@@ -4176,7 +4176,7 @@
       </c>
       <c r="P51">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="52" spans="1:16" x14ac:dyDescent="0.25">
@@ -4205,7 +4205,7 @@
         <v>10</v>
       </c>
       <c r="I52">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J52">
         <v>0</v>
@@ -4227,7 +4227,7 @@
       </c>
       <c r="P52">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="53" spans="1:16" x14ac:dyDescent="0.25">
@@ -4256,7 +4256,7 @@
         <v>10</v>
       </c>
       <c r="I53">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J53">
         <v>10</v>
@@ -4307,7 +4307,7 @@
         <v>10</v>
       </c>
       <c r="I54">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J54">
         <v>0</v>
@@ -4329,7 +4329,7 @@
       </c>
       <c r="P54">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="55" spans="1:16" x14ac:dyDescent="0.25">
@@ -4358,7 +4358,7 @@
         <v>10</v>
       </c>
       <c r="I55">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J55">
         <v>10</v>
@@ -4409,7 +4409,7 @@
         <v>10</v>
       </c>
       <c r="I56">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J56">
         <v>10</v>
@@ -4460,7 +4460,7 @@
         <v>10</v>
       </c>
       <c r="I57">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J57">
         <v>10</v>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="P57">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="58" spans="1:16" x14ac:dyDescent="0.25">
@@ -4511,7 +4511,7 @@
         <v>10</v>
       </c>
       <c r="I58">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J58">
         <v>10</v>
@@ -4533,7 +4533,7 @@
       </c>
       <c r="P58">
         <f t="shared" si="0"/>
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="59" spans="1:16" x14ac:dyDescent="0.25">
@@ -4562,7 +4562,7 @@
         <v>10</v>
       </c>
       <c r="I59">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J59">
         <v>0</v>
@@ -4584,7 +4584,7 @@
       </c>
       <c r="P59">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="60" spans="1:16" x14ac:dyDescent="0.25">
@@ -4613,7 +4613,7 @@
         <v>10</v>
       </c>
       <c r="I60">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J60">
         <v>10</v>
@@ -4635,7 +4635,7 @@
       </c>
       <c r="P60">
         <f t="shared" si="0"/>
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="61" spans="1:16" x14ac:dyDescent="0.25">
@@ -4664,7 +4664,7 @@
         <v>10</v>
       </c>
       <c r="I61">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J61">
         <v>10</v>
@@ -4686,7 +4686,7 @@
       </c>
       <c r="P61">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="62" spans="1:16" x14ac:dyDescent="0.25">
@@ -4715,7 +4715,7 @@
         <v>0</v>
       </c>
       <c r="I62">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J62">
         <v>0</v>
@@ -4766,7 +4766,7 @@
         <v>10</v>
       </c>
       <c r="I63">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J63">
         <v>10</v>
@@ -4817,7 +4817,7 @@
         <v>10</v>
       </c>
       <c r="I64">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J64">
         <v>10</v>
@@ -4868,7 +4868,7 @@
         <v>10</v>
       </c>
       <c r="I65">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J65">
         <v>10</v>
@@ -4890,7 +4890,7 @@
       </c>
       <c r="P65">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="66" spans="1:16" x14ac:dyDescent="0.25">
@@ -4919,7 +4919,7 @@
         <v>10</v>
       </c>
       <c r="I66">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J66">
         <v>10</v>
@@ -4970,7 +4970,7 @@
         <v>10</v>
       </c>
       <c r="I67">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J67">
         <v>10</v>
@@ -5021,7 +5021,7 @@
         <v>10</v>
       </c>
       <c r="I68">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J68">
         <v>10</v>
@@ -5072,7 +5072,7 @@
         <v>10</v>
       </c>
       <c r="I69">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J69">
         <v>10</v>
@@ -5094,7 +5094,7 @@
       </c>
       <c r="P69">
         <f t="shared" si="1"/>
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="70" spans="1:16" x14ac:dyDescent="0.25">
@@ -5123,7 +5123,7 @@
         <v>10</v>
       </c>
       <c r="I70">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J70">
         <v>0</v>
@@ -5145,7 +5145,7 @@
       </c>
       <c r="P70">
         <f t="shared" si="1"/>
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="71" spans="1:16" x14ac:dyDescent="0.25">
@@ -5174,7 +5174,7 @@
         <v>0</v>
       </c>
       <c r="I71">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J71">
         <v>0</v>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="P71">
         <f t="shared" si="1"/>
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="72" spans="1:16" x14ac:dyDescent="0.25">
@@ -5225,7 +5225,7 @@
         <v>10</v>
       </c>
       <c r="I72">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J72">
         <v>10</v>
@@ -5247,7 +5247,7 @@
       </c>
       <c r="P72">
         <f t="shared" si="1"/>
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizacion de notas primer modulo
</commit_message>
<xml_diff>
--- a/backend/database/Seguidores_Primer_Modulo.xlsx
+++ b/backend/database/Seguidores_Primer_Modulo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/24b0972e82577483/CLOUDGER/DOCKER/NOTAS_MOVI_APP/notasseguidores/app/backend/database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="49" documentId="8_{CB1EA7B0-2F00-435E-A2E5-997CDBADE84E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B223C419-B485-4544-838F-12A10B0266E9}"/>
+  <xr:revisionPtr revIDLastSave="54" documentId="8_{CB1EA7B0-2F00-435E-A2E5-997CDBADE84E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2FFF8A89-41AE-4187-A667-A525699756E7}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5BEBD1D6-3E86-4F2C-B143-CBE730185EB4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5BEBD1D6-3E86-4F2C-B143-CBE730185EB4}"/>
   </bookViews>
   <sheets>
     <sheet name="Seguidores_Primer_Modulo" sheetId="1" r:id="rId1"/>
@@ -705,7 +705,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -836,6 +836,14 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1138,7 +1146,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="42">
+  <cellStyleXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
@@ -1181,11 +1189,13 @@
     <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="42"/>
   </cellXfs>
-  <cellStyles count="42">
+  <cellStyles count="43">
     <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
     <cellStyle name="20% - Énfasis2" xfId="23" builtinId="34" customBuiltin="1"/>
     <cellStyle name="20% - Énfasis3" xfId="27" builtinId="38" customBuiltin="1"/>
@@ -1217,6 +1227,7 @@
     <cellStyle name="Énfasis5" xfId="34" builtinId="45" customBuiltin="1"/>
     <cellStyle name="Énfasis6" xfId="38" builtinId="49" customBuiltin="1"/>
     <cellStyle name="Entrada" xfId="9" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="Hipervínculo" xfId="42" builtinId="8"/>
     <cellStyle name="Incorrecto" xfId="7" builtinId="27" customBuiltin="1"/>
     <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1630,23 +1641,23 @@
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>9</v>
+      <c r="A2">
+        <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="C2" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="D2">
         <v>10</v>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G2">
         <v>10</v>
@@ -1667,28 +1678,28 @@
         <v>0</v>
       </c>
       <c r="M2">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P2">
         <f>ROUNDUP(AVERAGE(D2:O2),0)</f>
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>12</v>
+      <c r="A3">
+        <v>0</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>118</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
+        <v>119</v>
       </c>
       <c r="D3">
         <v>10</v>
@@ -1700,7 +1711,7 @@
         <v>10</v>
       </c>
       <c r="G3">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H3">
         <v>10</v>
@@ -1727,19 +1738,19 @@
         <v>10</v>
       </c>
       <c r="P3">
-        <f t="shared" ref="P3:P66" si="0">ROUNDUP(AVERAGE(D3:O3),0)</f>
-        <v>9</v>
+        <f>ROUNDUP(AVERAGE(D3:O3),0)</f>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>15</v>
+      <c r="A4">
+        <v>0</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>209</v>
       </c>
       <c r="C4" t="s">
-        <v>17</v>
+        <v>210</v>
       </c>
       <c r="D4">
         <v>10</v>
@@ -1754,13 +1765,13 @@
         <v>10</v>
       </c>
       <c r="H4">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="I4">
         <v>10</v>
       </c>
       <c r="J4">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K4">
         <v>10</v>
@@ -1772,25 +1783,25 @@
         <v>10</v>
       </c>
       <c r="N4">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="O4">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="P4">
-        <f t="shared" si="0"/>
-        <v>10</v>
+        <f>ROUNDUP(AVERAGE(D4:O4),0)</f>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>41</v>
       </c>
       <c r="C5" t="s">
-        <v>20</v>
+        <v>42</v>
       </c>
       <c r="D5">
         <v>10</v>
@@ -1814,7 +1825,7 @@
         <v>10</v>
       </c>
       <c r="K5">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="L5">
         <v>10</v>
@@ -1826,11 +1837,11 @@
         <v>10</v>
       </c>
       <c r="O5">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P5">
-        <f t="shared" si="0"/>
-        <v>9</v>
+        <f>ROUNDUP(AVERAGE(D5:O5),0)</f>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
@@ -1880,25 +1891,25 @@
         <v>0</v>
       </c>
       <c r="P6">
-        <f t="shared" si="0"/>
+        <f>ROUNDUP(AVERAGE(D6:O6),0)</f>
         <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>24</v>
+        <v>88</v>
       </c>
       <c r="B7" t="s">
-        <v>25</v>
+        <v>89</v>
       </c>
       <c r="C7" t="s">
-        <v>26</v>
+        <v>90</v>
       </c>
       <c r="D7">
         <v>10</v>
       </c>
       <c r="E7">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F7">
         <v>0</v>
@@ -1922,28 +1933,28 @@
         <v>10</v>
       </c>
       <c r="M7">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="N7">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="O7">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="P7">
-        <f t="shared" si="0"/>
-        <v>10</v>
+        <f>ROUNDUP(AVERAGE(D7:O7),0)</f>
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>27</v>
+        <v>126</v>
       </c>
       <c r="B8" t="s">
-        <v>28</v>
-      </c>
-      <c r="C8" t="s">
-        <v>29</v>
+        <v>127</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>128</v>
       </c>
       <c r="D8">
         <v>10</v>
@@ -1967,7 +1978,7 @@
         <v>10</v>
       </c>
       <c r="K8">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L8">
         <v>10</v>
@@ -1982,19 +1993,19 @@
         <v>10</v>
       </c>
       <c r="P8">
-        <f t="shared" si="0"/>
+        <f>ROUNDUP(AVERAGE(D8:O8),0)</f>
         <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>30</v>
+        <v>126</v>
       </c>
       <c r="B9" t="s">
-        <v>28</v>
+        <v>145</v>
       </c>
       <c r="C9" t="s">
-        <v>31</v>
+        <v>146</v>
       </c>
       <c r="D9">
         <v>10</v>
@@ -2024,28 +2035,28 @@
         <v>10</v>
       </c>
       <c r="M9">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="N9">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="O9">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P9">
-        <f t="shared" si="0"/>
-        <v>10</v>
+        <f>ROUNDUP(AVERAGE(D9:O9),0)</f>
+        <v>9</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A10">
-        <v>0</v>
+      <c r="A10" t="s">
+        <v>162</v>
       </c>
       <c r="B10" t="s">
-        <v>32</v>
+        <v>163</v>
       </c>
       <c r="C10" t="s">
-        <v>33</v>
+        <v>164</v>
       </c>
       <c r="D10">
         <v>10</v>
@@ -2072,7 +2083,7 @@
         <v>10</v>
       </c>
       <c r="L10">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M10">
         <v>10</v>
@@ -2084,25 +2095,25 @@
         <v>10</v>
       </c>
       <c r="P10">
-        <f t="shared" si="0"/>
+        <f>ROUNDUP(AVERAGE(D10:O10),0)</f>
         <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>34</v>
+        <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="C11" t="s">
-        <v>36</v>
+        <v>14</v>
       </c>
       <c r="D11">
         <v>10</v>
       </c>
       <c r="E11">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F11">
         <v>10</v>
@@ -2120,10 +2131,10 @@
         <v>10</v>
       </c>
       <c r="K11">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L11">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="M11">
         <v>10</v>
@@ -2132,22 +2143,22 @@
         <v>10</v>
       </c>
       <c r="O11">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P11">
-        <f t="shared" si="0"/>
+        <f>ROUNDUP(AVERAGE(D11:O11),0)</f>
         <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>37</v>
+        <v>168</v>
       </c>
       <c r="B12" t="s">
-        <v>38</v>
+        <v>169</v>
       </c>
       <c r="C12" t="s">
-        <v>39</v>
+        <v>170</v>
       </c>
       <c r="D12">
         <v>10</v>
@@ -2171,7 +2182,7 @@
         <v>10</v>
       </c>
       <c r="K12">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L12">
         <v>10</v>
@@ -2186,19 +2197,19 @@
         <v>10</v>
       </c>
       <c r="P12">
-        <f t="shared" si="0"/>
+        <f>ROUNDUP(AVERAGE(D12:O12),0)</f>
         <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>40</v>
+        <v>147</v>
       </c>
       <c r="B13" t="s">
-        <v>41</v>
+        <v>148</v>
       </c>
       <c r="C13" t="s">
-        <v>42</v>
+        <v>149</v>
       </c>
       <c r="D13">
         <v>10</v>
@@ -2234,22 +2245,22 @@
         <v>10</v>
       </c>
       <c r="O13">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P13">
-        <f t="shared" si="0"/>
+        <f>ROUNDUP(AVERAGE(D13:O13),0)</f>
         <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B14" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C14" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D14">
         <v>10</v>
@@ -2258,7 +2269,7 @@
         <v>10</v>
       </c>
       <c r="F14">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G14">
         <v>10</v>
@@ -2288,19 +2299,19 @@
         <v>10</v>
       </c>
       <c r="P14">
-        <f t="shared" si="0"/>
+        <f>ROUNDUP(AVERAGE(D14:O14),0)</f>
         <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="B15" t="s">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="C15" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="D15">
         <v>10</v>
@@ -2339,28 +2350,28 @@
         <v>10</v>
       </c>
       <c r="P15">
-        <f t="shared" si="0"/>
+        <f>ROUNDUP(AVERAGE(D15:O15),0)</f>
         <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="B16" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="C16" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="D16">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E16">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F16">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G16">
         <v>10</v>
@@ -2378,10 +2389,10 @@
         <v>10</v>
       </c>
       <c r="L16">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M16">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="N16">
         <v>0</v>
@@ -2390,19 +2401,19 @@
         <v>0</v>
       </c>
       <c r="P16">
-        <f t="shared" si="0"/>
-        <v>5</v>
+        <f>ROUNDUP(AVERAGE(D16:O16),0)</f>
+        <v>7</v>
       </c>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>52</v>
+        <v>188</v>
       </c>
       <c r="B17" t="s">
-        <v>53</v>
+        <v>189</v>
       </c>
       <c r="C17" t="s">
-        <v>54</v>
+        <v>190</v>
       </c>
       <c r="D17">
         <v>10</v>
@@ -2411,7 +2422,7 @@
         <v>10</v>
       </c>
       <c r="F17">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G17">
         <v>10</v>
@@ -2438,28 +2449,28 @@
         <v>10</v>
       </c>
       <c r="O17">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P17">
-        <f t="shared" si="0"/>
-        <v>9</v>
+        <f>ROUNDUP(AVERAGE(D17:O17),0)</f>
+        <v>10</v>
       </c>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>55</v>
+        <v>180</v>
       </c>
       <c r="B18" t="s">
-        <v>56</v>
+        <v>181</v>
       </c>
       <c r="C18" t="s">
-        <v>57</v>
+        <v>182</v>
       </c>
       <c r="D18">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="E18">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F18">
         <v>10</v>
@@ -2477,34 +2488,34 @@
         <v>10</v>
       </c>
       <c r="K18">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L18">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="M18">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="N18">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="O18">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="P18">
-        <f t="shared" si="0"/>
-        <v>10</v>
+        <f>ROUNDUP(AVERAGE(D18:O18),0)</f>
+        <v>5</v>
       </c>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>58</v>
+        <v>129</v>
       </c>
       <c r="B19" t="s">
-        <v>59</v>
+        <v>127</v>
       </c>
       <c r="C19" t="s">
-        <v>60</v>
+        <v>130</v>
       </c>
       <c r="D19">
         <v>10</v>
@@ -2525,43 +2536,43 @@
         <v>10</v>
       </c>
       <c r="J19">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K19">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L19">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="M19">
         <v>0</v>
       </c>
       <c r="N19">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O19">
         <v>0</v>
       </c>
       <c r="P19">
-        <f t="shared" si="0"/>
+        <f>ROUNDUP(AVERAGE(D19:O19),0)</f>
         <v>7</v>
       </c>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="B20" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="C20" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="D20">
         <v>10</v>
       </c>
       <c r="E20">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F20">
         <v>10</v>
@@ -2576,13 +2587,13 @@
         <v>10</v>
       </c>
       <c r="J20">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K20">
         <v>10</v>
       </c>
       <c r="L20">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="M20">
         <v>10</v>
@@ -2591,22 +2602,22 @@
         <v>10</v>
       </c>
       <c r="O20">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="P20">
-        <f t="shared" si="0"/>
-        <v>10</v>
+        <f>ROUNDUP(AVERAGE(D20:O20),0)</f>
+        <v>8</v>
       </c>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>64</v>
+        <v>153</v>
       </c>
       <c r="B21" t="s">
-        <v>65</v>
+        <v>154</v>
       </c>
       <c r="C21" t="s">
-        <v>66</v>
+        <v>155</v>
       </c>
       <c r="D21">
         <v>10</v>
@@ -2621,7 +2632,7 @@
         <v>10</v>
       </c>
       <c r="H21">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I21">
         <v>10</v>
@@ -2630,13 +2641,13 @@
         <v>0</v>
       </c>
       <c r="K21">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L21">
         <v>0</v>
       </c>
       <c r="M21">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N21">
         <v>0</v>
@@ -2645,25 +2656,25 @@
         <v>0</v>
       </c>
       <c r="P21">
-        <f t="shared" si="0"/>
-        <v>4</v>
+        <f>ROUNDUP(AVERAGE(D21:O21),0)</f>
+        <v>6</v>
       </c>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B22" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C22" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D22">
         <v>10</v>
       </c>
       <c r="E22">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F22">
         <v>10</v>
@@ -2672,7 +2683,7 @@
         <v>10</v>
       </c>
       <c r="H22">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="I22">
         <v>10</v>
@@ -2681,34 +2692,34 @@
         <v>0</v>
       </c>
       <c r="K22">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L22">
         <v>0</v>
       </c>
       <c r="M22">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="N22">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="O22">
         <v>0</v>
       </c>
       <c r="P22">
-        <f t="shared" si="0"/>
-        <v>8</v>
+        <f>ROUNDUP(AVERAGE(D22:O22),0)</f>
+        <v>4</v>
       </c>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="B23" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="C23" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="D23">
         <v>10</v>
@@ -2717,7 +2728,7 @@
         <v>0</v>
       </c>
       <c r="F23">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G23">
         <v>10</v>
@@ -2732,40 +2743,40 @@
         <v>10</v>
       </c>
       <c r="K23">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L23">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M23">
         <v>10</v>
       </c>
       <c r="N23">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O23">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P23">
-        <f t="shared" si="0"/>
-        <v>5</v>
+        <f>ROUNDUP(AVERAGE(D23:O23),0)</f>
+        <v>10</v>
       </c>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>73</v>
+        <v>191</v>
       </c>
       <c r="B24" t="s">
-        <v>74</v>
+        <v>192</v>
       </c>
       <c r="C24" t="s">
-        <v>75</v>
+        <v>193</v>
       </c>
       <c r="D24">
         <v>10</v>
       </c>
       <c r="E24">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F24">
         <v>10</v>
@@ -2798,79 +2809,79 @@
         <v>10</v>
       </c>
       <c r="P24">
-        <f t="shared" si="0"/>
+        <f>ROUNDUP(AVERAGE(D24:O24),0)</f>
         <v>10</v>
       </c>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>76</v>
+        <v>18</v>
       </c>
       <c r="B25" t="s">
-        <v>77</v>
+        <v>19</v>
       </c>
       <c r="C25" t="s">
-        <v>78</v>
+        <v>20</v>
       </c>
       <c r="D25">
         <v>10</v>
       </c>
       <c r="E25">
+        <v>10</v>
+      </c>
+      <c r="F25">
+        <v>10</v>
+      </c>
+      <c r="G25">
+        <v>10</v>
+      </c>
+      <c r="H25">
+        <v>10</v>
+      </c>
+      <c r="I25">
+        <v>10</v>
+      </c>
+      <c r="J25">
+        <v>10</v>
+      </c>
+      <c r="K25">
+        <v>7</v>
+      </c>
+      <c r="L25">
+        <v>10</v>
+      </c>
+      <c r="M25">
+        <v>10</v>
+      </c>
+      <c r="N25">
+        <v>10</v>
+      </c>
+      <c r="O25">
+        <v>0</v>
+      </c>
+      <c r="P25">
+        <f>ROUNDUP(AVERAGE(D25:O25),0)</f>
         <v>9</v>
-      </c>
-      <c r="F25">
-        <v>10</v>
-      </c>
-      <c r="G25">
-        <v>10</v>
-      </c>
-      <c r="H25">
-        <v>10</v>
-      </c>
-      <c r="I25">
-        <v>10</v>
-      </c>
-      <c r="J25">
-        <v>10</v>
-      </c>
-      <c r="K25">
-        <v>10</v>
-      </c>
-      <c r="L25">
-        <v>10</v>
-      </c>
-      <c r="M25">
-        <v>10</v>
-      </c>
-      <c r="N25">
-        <v>10</v>
-      </c>
-      <c r="O25">
-        <v>10</v>
-      </c>
-      <c r="P25">
-        <f t="shared" si="0"/>
-        <v>10</v>
       </c>
     </row>
     <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>79</v>
+        <v>100</v>
       </c>
       <c r="B26" t="s">
-        <v>80</v>
+        <v>101</v>
       </c>
       <c r="C26" t="s">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="D26">
         <v>10</v>
       </c>
       <c r="E26">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F26">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G26">
         <v>10</v>
@@ -2891,34 +2902,34 @@
         <v>10</v>
       </c>
       <c r="M26">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="N26">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="O26">
         <v>0</v>
       </c>
       <c r="P26">
-        <f t="shared" si="0"/>
+        <f>ROUNDUP(AVERAGE(D26:O26),0)</f>
         <v>9</v>
       </c>
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>82</v>
+        <v>185</v>
       </c>
       <c r="B27" t="s">
-        <v>83</v>
+        <v>186</v>
       </c>
       <c r="C27" t="s">
-        <v>84</v>
+        <v>187</v>
       </c>
       <c r="D27">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E27">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F27">
         <v>10</v>
@@ -2951,22 +2962,22 @@
         <v>10</v>
       </c>
       <c r="P27">
-        <f t="shared" si="0"/>
+        <f>ROUNDUP(AVERAGE(D27:O27),0)</f>
         <v>10</v>
       </c>
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>85</v>
+        <v>139</v>
       </c>
       <c r="B28" t="s">
-        <v>86</v>
+        <v>140</v>
       </c>
       <c r="C28" t="s">
-        <v>87</v>
+        <v>141</v>
       </c>
       <c r="D28">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="E28">
         <v>10</v>
@@ -2987,13 +2998,13 @@
         <v>10</v>
       </c>
       <c r="K28">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L28">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="M28">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="N28">
         <v>0</v>
@@ -3002,46 +3013,46 @@
         <v>0</v>
       </c>
       <c r="P28">
-        <f t="shared" si="0"/>
-        <v>9</v>
+        <f>ROUNDUP(AVERAGE(D28:O28),0)</f>
+        <v>5</v>
       </c>
     </row>
     <row r="29" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>88</v>
+        <v>136</v>
       </c>
       <c r="B29" t="s">
-        <v>89</v>
+        <v>137</v>
       </c>
       <c r="C29" t="s">
-        <v>90</v>
+        <v>138</v>
       </c>
       <c r="D29">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="E29">
         <v>0</v>
       </c>
       <c r="F29">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G29">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H29">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="I29">
         <v>10</v>
       </c>
       <c r="J29">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K29">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L29">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="M29">
         <v>0</v>
@@ -3053,31 +3064,31 @@
         <v>0</v>
       </c>
       <c r="P29">
-        <f t="shared" si="0"/>
-        <v>6</v>
+        <f>ROUNDUP(AVERAGE(D29:O29),0)</f>
+        <v>2</v>
       </c>
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="B30" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="C30" t="s">
-        <v>93</v>
+        <v>84</v>
       </c>
       <c r="D30">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E30">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F30">
         <v>10</v>
       </c>
       <c r="G30">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H30">
         <v>10</v>
@@ -3086,7 +3097,7 @@
         <v>10</v>
       </c>
       <c r="J30">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K30">
         <v>10</v>
@@ -3095,28 +3106,28 @@
         <v>10</v>
       </c>
       <c r="M30">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N30">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O30">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P30">
-        <f t="shared" si="0"/>
-        <v>6</v>
+        <f>ROUNDUP(AVERAGE(D30:O30),0)</f>
+        <v>10</v>
       </c>
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>94</v>
+        <v>203</v>
       </c>
       <c r="B31" t="s">
-        <v>95</v>
+        <v>204</v>
       </c>
       <c r="C31" t="s">
-        <v>96</v>
+        <v>205</v>
       </c>
       <c r="D31">
         <v>10</v>
@@ -3125,7 +3136,7 @@
         <v>10</v>
       </c>
       <c r="F31">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="G31">
         <v>10</v>
@@ -3146,34 +3157,34 @@
         <v>10</v>
       </c>
       <c r="M31">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="N31">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="O31">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="P31">
-        <f t="shared" si="0"/>
-        <v>10</v>
+        <f>ROUNDUP(AVERAGE(D31:O31),0)</f>
+        <v>7</v>
       </c>
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B32" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C32" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="D32">
         <v>10</v>
       </c>
       <c r="E32">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F32">
         <v>10</v>
@@ -3200,25 +3211,25 @@
         <v>10</v>
       </c>
       <c r="N32">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="O32">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="P32">
-        <f t="shared" si="0"/>
-        <v>9</v>
+        <f>ROUNDUP(AVERAGE(D32:O32),0)</f>
+        <v>10</v>
       </c>
     </row>
     <row r="33" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>100</v>
+        <v>165</v>
       </c>
       <c r="B33" t="s">
-        <v>101</v>
+        <v>166</v>
       </c>
       <c r="C33" t="s">
-        <v>102</v>
+        <v>167</v>
       </c>
       <c r="D33">
         <v>10</v>
@@ -3248,28 +3259,28 @@
         <v>10</v>
       </c>
       <c r="M33">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N33">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="O33">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P33">
-        <f t="shared" si="0"/>
-        <v>9</v>
+        <f>ROUNDUP(AVERAGE(D33:O33),0)</f>
+        <v>10</v>
       </c>
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>103</v>
+        <v>24</v>
       </c>
       <c r="B34" t="s">
-        <v>104</v>
+        <v>25</v>
       </c>
       <c r="C34" t="s">
-        <v>105</v>
+        <v>26</v>
       </c>
       <c r="D34">
         <v>10</v>
@@ -3278,7 +3289,7 @@
         <v>10</v>
       </c>
       <c r="F34">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="G34">
         <v>10</v>
@@ -3308,25 +3319,25 @@
         <v>10</v>
       </c>
       <c r="P34">
-        <f t="shared" si="0"/>
+        <f>ROUNDUP(AVERAGE(D34:O34),0)</f>
         <v>10</v>
       </c>
     </row>
     <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>106</v>
+        <v>76</v>
       </c>
       <c r="B35" t="s">
-        <v>107</v>
+        <v>77</v>
       </c>
       <c r="C35" t="s">
-        <v>108</v>
+        <v>78</v>
       </c>
       <c r="D35">
         <v>10</v>
       </c>
       <c r="E35">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F35">
         <v>10</v>
@@ -3359,19 +3370,19 @@
         <v>10</v>
       </c>
       <c r="P35">
-        <f t="shared" si="0"/>
+        <f>ROUNDUP(AVERAGE(D35:O35),0)</f>
         <v>10</v>
       </c>
     </row>
     <row r="36" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>109</v>
+        <v>174</v>
       </c>
       <c r="B36" t="s">
-        <v>110</v>
+        <v>175</v>
       </c>
       <c r="C36" t="s">
-        <v>111</v>
+        <v>176</v>
       </c>
       <c r="D36">
         <v>10</v>
@@ -3383,7 +3394,7 @@
         <v>10</v>
       </c>
       <c r="G36">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H36">
         <v>10</v>
@@ -3392,37 +3403,37 @@
         <v>10</v>
       </c>
       <c r="J36">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K36">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L36">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="M36">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="N36">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="O36">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="P36">
-        <f t="shared" si="0"/>
-        <v>10</v>
+        <f>ROUNDUP(AVERAGE(D36:O36),0)</f>
+        <v>5</v>
       </c>
     </row>
     <row r="37" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="B37" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="C37" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="D37">
         <v>10</v>
@@ -3461,25 +3472,25 @@
         <v>10</v>
       </c>
       <c r="P37">
-        <f t="shared" si="0"/>
+        <f>ROUNDUP(AVERAGE(D37:O37),0)</f>
         <v>10</v>
       </c>
     </row>
     <row r="38" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>115</v>
+        <v>171</v>
       </c>
       <c r="B38" t="s">
-        <v>116</v>
+        <v>172</v>
       </c>
       <c r="C38" t="s">
-        <v>117</v>
+        <v>173</v>
       </c>
       <c r="D38">
         <v>10</v>
       </c>
       <c r="E38">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F38">
         <v>10</v>
@@ -3500,31 +3511,31 @@
         <v>10</v>
       </c>
       <c r="L38">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M38">
         <v>0</v>
       </c>
       <c r="N38">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="O38">
         <v>0</v>
       </c>
       <c r="P38">
-        <f t="shared" si="0"/>
-        <v>7</v>
+        <f>ROUNDUP(AVERAGE(D38:O38),0)</f>
+        <v>8</v>
       </c>
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A39">
-        <v>0</v>
+      <c r="A39" t="s">
+        <v>73</v>
       </c>
       <c r="B39" t="s">
-        <v>118</v>
+        <v>74</v>
       </c>
       <c r="C39" t="s">
-        <v>119</v>
+        <v>75</v>
       </c>
       <c r="D39">
         <v>10</v>
@@ -3536,7 +3547,7 @@
         <v>10</v>
       </c>
       <c r="G39">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H39">
         <v>10</v>
@@ -3548,10 +3559,10 @@
         <v>10</v>
       </c>
       <c r="K39">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L39">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M39">
         <v>10</v>
@@ -3563,19 +3574,19 @@
         <v>10</v>
       </c>
       <c r="P39">
-        <f t="shared" si="0"/>
-        <v>8</v>
+        <f>ROUNDUP(AVERAGE(D39:O39),0)</f>
+        <v>10</v>
       </c>
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>120</v>
+        <v>15</v>
       </c>
       <c r="B40" t="s">
-        <v>121</v>
+        <v>16</v>
       </c>
       <c r="C40" t="s">
-        <v>122</v>
+        <v>17</v>
       </c>
       <c r="D40">
         <v>10</v>
@@ -3614,19 +3625,19 @@
         <v>10</v>
       </c>
       <c r="P40">
-        <f t="shared" si="0"/>
+        <f>ROUNDUP(AVERAGE(D40:O40),0)</f>
         <v>10</v>
       </c>
     </row>
     <row r="41" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>123</v>
+        <v>106</v>
       </c>
       <c r="B41" t="s">
-        <v>124</v>
+        <v>107</v>
       </c>
       <c r="C41" t="s">
-        <v>125</v>
+        <v>108</v>
       </c>
       <c r="D41">
         <v>10</v>
@@ -3662,22 +3673,22 @@
         <v>10</v>
       </c>
       <c r="O41">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P41">
-        <f t="shared" si="0"/>
+        <f>ROUNDUP(AVERAGE(D41:O41),0)</f>
         <v>10</v>
       </c>
     </row>
     <row r="42" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>126</v>
+        <v>200</v>
       </c>
       <c r="B42" t="s">
-        <v>127</v>
+        <v>201</v>
       </c>
       <c r="C42" t="s">
-        <v>128</v>
+        <v>202</v>
       </c>
       <c r="D42">
         <v>10</v>
@@ -3701,7 +3712,7 @@
         <v>10</v>
       </c>
       <c r="K42">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L42">
         <v>10</v>
@@ -3716,19 +3727,19 @@
         <v>10</v>
       </c>
       <c r="P42">
-        <f t="shared" si="0"/>
+        <f>ROUNDUP(AVERAGE(D42:O42),0)</f>
         <v>10</v>
       </c>
     </row>
     <row r="43" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>129</v>
+        <v>27</v>
       </c>
       <c r="B43" t="s">
-        <v>127</v>
+        <v>28</v>
       </c>
       <c r="C43" t="s">
-        <v>130</v>
+        <v>29</v>
       </c>
       <c r="D43">
         <v>10</v>
@@ -3752,37 +3763,37 @@
         <v>10</v>
       </c>
       <c r="K43">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L43">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M43">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N43">
         <v>10</v>
       </c>
       <c r="O43">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P43">
-        <f t="shared" si="0"/>
-        <v>7</v>
+        <f>ROUNDUP(AVERAGE(D43:O43),0)</f>
+        <v>10</v>
       </c>
     </row>
     <row r="44" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>131</v>
+        <v>34</v>
       </c>
       <c r="B44" t="s">
-        <v>132</v>
+        <v>35</v>
       </c>
       <c r="C44" t="s">
-        <v>133</v>
+        <v>36</v>
       </c>
       <c r="D44">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E44">
         <v>0</v>
@@ -3818,19 +3829,19 @@
         <v>0</v>
       </c>
       <c r="P44">
-        <f t="shared" si="0"/>
-        <v>8</v>
+        <f>ROUNDUP(AVERAGE(D44:O44),0)</f>
+        <v>9</v>
       </c>
     </row>
     <row r="45" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>131</v>
+        <v>79</v>
       </c>
       <c r="B45" t="s">
-        <v>134</v>
+        <v>80</v>
       </c>
       <c r="C45" t="s">
-        <v>135</v>
+        <v>81</v>
       </c>
       <c r="D45">
         <v>10</v>
@@ -3839,7 +3850,7 @@
         <v>0</v>
       </c>
       <c r="F45">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G45">
         <v>10</v>
@@ -3869,73 +3880,73 @@
         <v>0</v>
       </c>
       <c r="P45">
-        <f t="shared" si="0"/>
+        <f>ROUNDUP(AVERAGE(D45:O45),0)</f>
         <v>9</v>
       </c>
     </row>
     <row r="46" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>136</v>
+        <v>123</v>
       </c>
       <c r="B46" t="s">
-        <v>137</v>
-      </c>
-      <c r="C46" t="s">
-        <v>138</v>
+        <v>124</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>125</v>
       </c>
       <c r="D46">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E46">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F46">
         <v>10</v>
       </c>
       <c r="G46">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H46">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I46">
         <v>10</v>
       </c>
       <c r="J46">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K46">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L46">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M46">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N46">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O46">
         <v>0</v>
       </c>
       <c r="P46">
-        <f t="shared" si="0"/>
-        <v>2</v>
+        <f>ROUNDUP(AVERAGE(D46:O46),0)</f>
+        <v>10</v>
       </c>
     </row>
     <row r="47" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>139</v>
+        <v>112</v>
       </c>
       <c r="B47" t="s">
-        <v>140</v>
+        <v>113</v>
       </c>
       <c r="C47" t="s">
-        <v>141</v>
+        <v>114</v>
       </c>
       <c r="D47">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E47">
         <v>10</v>
@@ -3956,23 +3967,23 @@
         <v>10</v>
       </c>
       <c r="K47">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L47">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M47">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N47">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O47">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P47">
-        <f t="shared" si="0"/>
-        <v>5</v>
+        <f>ROUNDUP(AVERAGE(D47:O47),0)</f>
+        <v>10</v>
       </c>
     </row>
     <row r="48" spans="1:16" x14ac:dyDescent="0.25">
@@ -4022,19 +4033,19 @@
         <v>10</v>
       </c>
       <c r="P48">
-        <f t="shared" si="0"/>
+        <f>ROUNDUP(AVERAGE(D48:O48),0)</f>
         <v>10</v>
       </c>
     </row>
     <row r="49" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>126</v>
+        <v>91</v>
       </c>
       <c r="B49" t="s">
-        <v>145</v>
+        <v>92</v>
       </c>
       <c r="C49" t="s">
-        <v>146</v>
+        <v>93</v>
       </c>
       <c r="D49">
         <v>10</v>
@@ -4046,7 +4057,7 @@
         <v>10</v>
       </c>
       <c r="G49">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H49">
         <v>10</v>
@@ -4055,7 +4066,7 @@
         <v>10</v>
       </c>
       <c r="J49">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K49">
         <v>10</v>
@@ -4070,22 +4081,22 @@
         <v>0</v>
       </c>
       <c r="O49">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="P49">
-        <f t="shared" si="0"/>
-        <v>9</v>
+        <f>ROUNDUP(AVERAGE(D49:O49),0)</f>
+        <v>6</v>
       </c>
     </row>
     <row r="50" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>147</v>
+        <v>52</v>
       </c>
       <c r="B50" t="s">
-        <v>148</v>
+        <v>53</v>
       </c>
       <c r="C50" t="s">
-        <v>149</v>
+        <v>54</v>
       </c>
       <c r="D50">
         <v>10</v>
@@ -4094,7 +4105,7 @@
         <v>10</v>
       </c>
       <c r="F50">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="G50">
         <v>10</v>
@@ -4121,31 +4132,31 @@
         <v>10</v>
       </c>
       <c r="O50">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="P50">
-        <f t="shared" si="0"/>
-        <v>10</v>
+        <f>ROUNDUP(AVERAGE(D50:O50),0)</f>
+        <v>9</v>
       </c>
     </row>
     <row r="51" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>150</v>
+        <v>9</v>
       </c>
       <c r="B51" t="s">
-        <v>151</v>
+        <v>10</v>
       </c>
       <c r="C51" t="s">
-        <v>152</v>
+        <v>11</v>
       </c>
       <c r="D51">
         <v>10</v>
       </c>
       <c r="E51">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F51">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="G51">
         <v>10</v>
@@ -4157,37 +4168,37 @@
         <v>10</v>
       </c>
       <c r="J51">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K51">
         <v>10</v>
       </c>
       <c r="L51">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="M51">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="N51">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="O51">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="P51">
-        <f t="shared" si="0"/>
-        <v>10</v>
+        <f>ROUNDUP(AVERAGE(D51:O51),0)</f>
+        <v>5</v>
       </c>
     </row>
     <row r="52" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>153</v>
+        <v>115</v>
       </c>
       <c r="B52" t="s">
-        <v>154</v>
+        <v>116</v>
       </c>
       <c r="C52" t="s">
-        <v>155</v>
+        <v>117</v>
       </c>
       <c r="D52">
         <v>10</v>
@@ -4208,7 +4219,7 @@
         <v>10</v>
       </c>
       <c r="J52">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K52">
         <v>10</v>
@@ -4217,34 +4228,34 @@
         <v>0</v>
       </c>
       <c r="M52">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="N52">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O52">
         <v>0</v>
       </c>
       <c r="P52">
-        <f t="shared" si="0"/>
-        <v>6</v>
+        <f>ROUNDUP(AVERAGE(D52:O52),0)</f>
+        <v>7</v>
       </c>
     </row>
     <row r="53" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>156</v>
+        <v>131</v>
       </c>
       <c r="B53" t="s">
-        <v>157</v>
+        <v>132</v>
       </c>
       <c r="C53" t="s">
-        <v>158</v>
+        <v>133</v>
       </c>
       <c r="D53">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E53">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F53">
         <v>10</v>
@@ -4274,34 +4285,34 @@
         <v>10</v>
       </c>
       <c r="O53">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="P53">
-        <f t="shared" si="0"/>
-        <v>10</v>
+        <f>ROUNDUP(AVERAGE(D53:O53),0)</f>
+        <v>8</v>
       </c>
     </row>
     <row r="54" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>159</v>
+        <v>131</v>
       </c>
       <c r="B54" t="s">
-        <v>160</v>
+        <v>134</v>
       </c>
       <c r="C54" t="s">
-        <v>161</v>
+        <v>135</v>
       </c>
       <c r="D54">
         <v>10</v>
       </c>
       <c r="E54">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F54">
         <v>10</v>
       </c>
       <c r="G54">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H54">
         <v>10</v>
@@ -4310,7 +4321,7 @@
         <v>10</v>
       </c>
       <c r="J54">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K54">
         <v>10</v>
@@ -4325,31 +4336,31 @@
         <v>10</v>
       </c>
       <c r="O54">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="P54">
-        <f t="shared" si="0"/>
+        <f>ROUNDUP(AVERAGE(D54:O54),0)</f>
         <v>9</v>
       </c>
     </row>
     <row r="55" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>162</v>
+        <v>70</v>
       </c>
       <c r="B55" t="s">
-        <v>163</v>
+        <v>71</v>
       </c>
       <c r="C55" t="s">
-        <v>164</v>
+        <v>72</v>
       </c>
       <c r="D55">
         <v>10</v>
       </c>
       <c r="E55">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F55">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="G55">
         <v>10</v>
@@ -4364,43 +4375,43 @@
         <v>10</v>
       </c>
       <c r="K55">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L55">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="M55">
         <v>10</v>
       </c>
       <c r="N55">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="O55">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="P55">
-        <f t="shared" si="0"/>
-        <v>10</v>
+        <f>ROUNDUP(AVERAGE(D55:O55),0)</f>
+        <v>5</v>
       </c>
     </row>
     <row r="56" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>165</v>
+        <v>177</v>
       </c>
       <c r="B56" t="s">
-        <v>166</v>
+        <v>178</v>
       </c>
       <c r="C56" t="s">
-        <v>167</v>
+        <v>179</v>
       </c>
       <c r="D56">
         <v>10</v>
       </c>
       <c r="E56">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F56">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="G56">
         <v>10</v>
@@ -4418,7 +4429,7 @@
         <v>10</v>
       </c>
       <c r="L56">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="M56">
         <v>10</v>
@@ -4427,22 +4438,22 @@
         <v>10</v>
       </c>
       <c r="O56">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="P56">
-        <f t="shared" si="0"/>
-        <v>10</v>
+        <f>ROUNDUP(AVERAGE(D56:O56),0)</f>
+        <v>8</v>
       </c>
     </row>
     <row r="57" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>168</v>
+        <v>85</v>
       </c>
       <c r="B57" t="s">
-        <v>169</v>
+        <v>86</v>
       </c>
       <c r="C57" t="s">
-        <v>170</v>
+        <v>87</v>
       </c>
       <c r="D57">
         <v>10</v>
@@ -4466,7 +4477,7 @@
         <v>10</v>
       </c>
       <c r="K57">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L57">
         <v>10</v>
@@ -4475,25 +4486,25 @@
         <v>10</v>
       </c>
       <c r="N57">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="O57">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="P57">
-        <f t="shared" si="0"/>
-        <v>10</v>
+        <f>ROUNDUP(AVERAGE(D57:O57),0)</f>
+        <v>9</v>
       </c>
     </row>
     <row r="58" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>171</v>
+        <v>156</v>
       </c>
       <c r="B58" t="s">
-        <v>172</v>
+        <v>157</v>
       </c>
       <c r="C58" t="s">
-        <v>173</v>
+        <v>158</v>
       </c>
       <c r="D58">
         <v>10</v>
@@ -4523,28 +4534,28 @@
         <v>10</v>
       </c>
       <c r="M58">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N58">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O58">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P58">
-        <f t="shared" si="0"/>
-        <v>8</v>
+        <f>ROUNDUP(AVERAGE(D58:O58),0)</f>
+        <v>10</v>
       </c>
     </row>
     <row r="59" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>174</v>
+        <v>206</v>
       </c>
       <c r="B59" t="s">
-        <v>175</v>
+        <v>207</v>
       </c>
       <c r="C59" t="s">
-        <v>176</v>
+        <v>208</v>
       </c>
       <c r="D59">
         <v>10</v>
@@ -4556,7 +4567,7 @@
         <v>10</v>
       </c>
       <c r="G59">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H59">
         <v>10</v>
@@ -4568,34 +4579,34 @@
         <v>0</v>
       </c>
       <c r="K59">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L59">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M59">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N59">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O59">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P59">
-        <f t="shared" si="0"/>
-        <v>5</v>
+        <f>ROUNDUP(AVERAGE(D59:O59),0)</f>
+        <v>10</v>
       </c>
     </row>
     <row r="60" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>177</v>
+        <v>97</v>
       </c>
       <c r="B60" t="s">
-        <v>178</v>
+        <v>98</v>
       </c>
       <c r="C60" t="s">
-        <v>179</v>
+        <v>99</v>
       </c>
       <c r="D60">
         <v>10</v>
@@ -4604,7 +4615,7 @@
         <v>0</v>
       </c>
       <c r="F60">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G60">
         <v>10</v>
@@ -4622,31 +4633,31 @@
         <v>10</v>
       </c>
       <c r="L60">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="M60">
         <v>10</v>
       </c>
       <c r="N60">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="O60">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="P60">
-        <f t="shared" si="0"/>
-        <v>8</v>
+        <f>ROUNDUP(AVERAGE(D60:O60),0)</f>
+        <v>9</v>
       </c>
     </row>
     <row r="61" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>180</v>
+        <v>49</v>
       </c>
       <c r="B61" t="s">
-        <v>181</v>
+        <v>50</v>
       </c>
       <c r="C61" t="s">
-        <v>182</v>
+        <v>51</v>
       </c>
       <c r="D61">
         <v>0</v>
@@ -4655,7 +4666,7 @@
         <v>0</v>
       </c>
       <c r="F61">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="G61">
         <v>10</v>
@@ -4667,16 +4678,16 @@
         <v>10</v>
       </c>
       <c r="J61">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K61">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L61">
         <v>0</v>
       </c>
       <c r="M61">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N61">
         <v>0</v>
@@ -4685,7 +4696,7 @@
         <v>0</v>
       </c>
       <c r="P61">
-        <f t="shared" si="0"/>
+        <f>ROUNDUP(AVERAGE(D61:O61),0)</f>
         <v>5</v>
       </c>
     </row>
@@ -4736,19 +4747,19 @@
         <v>10</v>
       </c>
       <c r="P62">
-        <f t="shared" si="0"/>
+        <f>ROUNDUP(AVERAGE(D62:O62),0)</f>
         <v>5</v>
       </c>
     </row>
     <row r="63" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>185</v>
+        <v>150</v>
       </c>
       <c r="B63" t="s">
-        <v>186</v>
+        <v>151</v>
       </c>
       <c r="C63" t="s">
-        <v>187</v>
+        <v>152</v>
       </c>
       <c r="D63">
         <v>10</v>
@@ -4769,7 +4780,7 @@
         <v>10</v>
       </c>
       <c r="J63">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K63">
         <v>10</v>
@@ -4787,19 +4798,19 @@
         <v>10</v>
       </c>
       <c r="P63">
-        <f t="shared" si="0"/>
+        <f>ROUNDUP(AVERAGE(D63:O63),0)</f>
         <v>10</v>
       </c>
     </row>
     <row r="64" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="B64" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="C64" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="D64">
         <v>10</v>
@@ -4838,28 +4849,28 @@
         <v>10</v>
       </c>
       <c r="P64">
-        <f t="shared" si="0"/>
+        <f>ROUNDUP(AVERAGE(D64:O64),0)</f>
         <v>10</v>
       </c>
     </row>
     <row r="65" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>191</v>
+        <v>43</v>
       </c>
       <c r="B65" t="s">
-        <v>192</v>
+        <v>44</v>
       </c>
       <c r="C65" t="s">
-        <v>193</v>
+        <v>45</v>
       </c>
       <c r="D65">
         <v>10</v>
       </c>
       <c r="E65">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F65">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="G65">
         <v>10</v>
@@ -4889,19 +4900,19 @@
         <v>10</v>
       </c>
       <c r="P65">
-        <f t="shared" si="0"/>
+        <f>ROUNDUP(AVERAGE(D65:O65),0)</f>
         <v>10</v>
       </c>
     </row>
     <row r="66" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>194</v>
+        <v>37</v>
       </c>
       <c r="B66" t="s">
-        <v>195</v>
+        <v>38</v>
       </c>
       <c r="C66" t="s">
-        <v>196</v>
+        <v>39</v>
       </c>
       <c r="D66">
         <v>10</v>
@@ -4940,19 +4951,19 @@
         <v>10</v>
       </c>
       <c r="P66">
-        <f t="shared" si="0"/>
+        <f>ROUNDUP(AVERAGE(D66:O66),0)</f>
         <v>10</v>
       </c>
     </row>
     <row r="67" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>197</v>
+        <v>30</v>
       </c>
       <c r="B67" t="s">
-        <v>198</v>
+        <v>28</v>
       </c>
       <c r="C67" t="s">
-        <v>199</v>
+        <v>31</v>
       </c>
       <c r="D67">
         <v>10</v>
@@ -4991,19 +5002,19 @@
         <v>10</v>
       </c>
       <c r="P67">
-        <f t="shared" ref="P67:P72" si="1">ROUNDUP(AVERAGE(D67:O67),0)</f>
+        <f>ROUNDUP(AVERAGE(D67:O67),0)</f>
         <v>10</v>
       </c>
     </row>
     <row r="68" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="B68" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="C68" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="D68">
         <v>10</v>
@@ -5042,28 +5053,28 @@
         <v>10</v>
       </c>
       <c r="P68">
-        <f t="shared" si="1"/>
+        <f>ROUNDUP(AVERAGE(D68:O68),0)</f>
         <v>10</v>
       </c>
     </row>
     <row r="69" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
       <c r="B69" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="C69" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="D69">
         <v>10</v>
       </c>
       <c r="E69">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F69">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G69">
         <v>10</v>
@@ -5084,28 +5095,28 @@
         <v>10</v>
       </c>
       <c r="M69">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N69">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O69">
         <v>0</v>
       </c>
       <c r="P69">
-        <f t="shared" si="1"/>
-        <v>7</v>
+        <f>ROUNDUP(AVERAGE(D69:O69),0)</f>
+        <v>9</v>
       </c>
     </row>
     <row r="70" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>206</v>
+        <v>159</v>
       </c>
       <c r="B70" t="s">
-        <v>207</v>
+        <v>160</v>
       </c>
       <c r="C70" t="s">
-        <v>208</v>
+        <v>161</v>
       </c>
       <c r="D70">
         <v>10</v>
@@ -5117,7 +5128,7 @@
         <v>10</v>
       </c>
       <c r="G70">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H70">
         <v>10</v>
@@ -5144,19 +5155,19 @@
         <v>10</v>
       </c>
       <c r="P70">
-        <f t="shared" si="1"/>
-        <v>10</v>
+        <f>ROUNDUP(AVERAGE(D70:O70),0)</f>
+        <v>9</v>
       </c>
     </row>
     <row r="71" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A71">
-        <v>0</v>
+      <c r="A71" t="s">
+        <v>109</v>
       </c>
       <c r="B71" t="s">
-        <v>209</v>
+        <v>110</v>
       </c>
       <c r="C71" t="s">
-        <v>210</v>
+        <v>111</v>
       </c>
       <c r="D71">
         <v>10</v>
@@ -5171,13 +5182,13 @@
         <v>10</v>
       </c>
       <c r="H71">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I71">
         <v>10</v>
       </c>
       <c r="J71">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K71">
         <v>10</v>
@@ -5189,31 +5200,31 @@
         <v>10</v>
       </c>
       <c r="N71">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O71">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P71">
-        <f t="shared" si="1"/>
-        <v>7</v>
+        <f>ROUNDUP(AVERAGE(D71:O71),0)</f>
+        <v>10</v>
       </c>
     </row>
     <row r="72" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>211</v>
+        <v>103</v>
       </c>
       <c r="B72" t="s">
-        <v>212</v>
+        <v>104</v>
       </c>
       <c r="C72" t="s">
-        <v>213</v>
+        <v>105</v>
       </c>
       <c r="D72">
         <v>10</v>
       </c>
       <c r="E72">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F72">
         <v>10</v>
@@ -5243,15 +5254,23 @@
         <v>10</v>
       </c>
       <c r="O72">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P72">
-        <f t="shared" si="1"/>
-        <v>9</v>
+        <f>ROUNDUP(AVERAGE(D72:O72),0)</f>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P72" xr:uid="{2AC72954-4A29-4392-87CA-18CD68D9BE96}"/>
+  <autoFilter ref="A1:P72" xr:uid="{2AC72954-4A29-4392-87CA-18CD68D9BE96}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:P72">
+      <sortCondition ref="A1:A72"/>
+    </sortState>
+  </autoFilter>
+  <hyperlinks>
+    <hyperlink ref="C46" r:id="rId1" xr:uid="{A84EDFBB-A320-47C6-8C70-A4E257E89128}"/>
+    <hyperlink ref="C8" r:id="rId2" xr:uid="{3E6984B4-6D6D-413D-9C0D-C499F9F2402E}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>